<commit_message>
Estimate loads for '002-1638-R'
</commit_message>
<xml_diff>
--- a/data/annual_loads_waterbodies.xlsx
+++ b/data/annual_loads_waterbodies.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F173"/>
+  <dimension ref="A1:F197"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4185,6 +4185,530 @@
       </c>
       <c r="F173" t="n">
         <v>195.5887791075585</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>002-1638-R</t>
+        </is>
+      </c>
+      <c r="B174" t="n">
+        <v>1995</v>
+      </c>
+      <c r="C174" t="n">
+        <v>216.5177960450953</v>
+      </c>
+      <c r="D174" t="n">
+        <v>6.619594004249908</v>
+      </c>
+      <c r="E174" t="n">
+        <v>3180.144565744456</v>
+      </c>
+      <c r="F174" t="n">
+        <v>948.6323535620309</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>002-1638-R</t>
+        </is>
+      </c>
+      <c r="B175" t="n">
+        <v>1996</v>
+      </c>
+      <c r="C175" t="n">
+        <v>205.1468362375021</v>
+      </c>
+      <c r="D175" t="n">
+        <v>6.883637384149339</v>
+      </c>
+      <c r="E175" t="n">
+        <v>2962.508476689706</v>
+      </c>
+      <c r="F175" t="n">
+        <v>676.6893552491267</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>002-1638-R</t>
+        </is>
+      </c>
+      <c r="B176" t="n">
+        <v>1997</v>
+      </c>
+      <c r="C176" t="n">
+        <v>195.083291129695</v>
+      </c>
+      <c r="D176" t="n">
+        <v>5.854821297076653</v>
+      </c>
+      <c r="E176" t="n">
+        <v>2791.367670829393</v>
+      </c>
+      <c r="F176" t="n">
+        <v>703.1272190033927</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>002-1638-R</t>
+        </is>
+      </c>
+      <c r="B177" t="n">
+        <v>1998</v>
+      </c>
+      <c r="C177" t="n">
+        <v>220.9255626131536</v>
+      </c>
+      <c r="D177" t="n">
+        <v>11.90320330132592</v>
+      </c>
+      <c r="E177" t="n">
+        <v>4949.10850836039</v>
+      </c>
+      <c r="F177" t="n">
+        <v>1007.593700058762</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>002-1638-R</t>
+        </is>
+      </c>
+      <c r="B178" t="n">
+        <v>1999</v>
+      </c>
+      <c r="C178" t="n">
+        <v>230.4513182461515</v>
+      </c>
+      <c r="D178" t="n">
+        <v>8.145762072400846</v>
+      </c>
+      <c r="E178" t="n">
+        <v>3266.478783973206</v>
+      </c>
+      <c r="F178" t="n">
+        <v>1219.598775148054</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>002-1638-R</t>
+        </is>
+      </c>
+      <c r="B179" t="n">
+        <v>2000</v>
+      </c>
+      <c r="C179" t="n">
+        <v>342.9725171733232</v>
+      </c>
+      <c r="D179" t="n">
+        <v>18.49844416800313</v>
+      </c>
+      <c r="E179" t="n">
+        <v>9754.12962479929</v>
+      </c>
+      <c r="F179" t="n">
+        <v>2126.151506620473</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>002-1638-R</t>
+        </is>
+      </c>
+      <c r="B180" t="n">
+        <v>2001</v>
+      </c>
+      <c r="C180" t="n">
+        <v>224.7186003443967</v>
+      </c>
+      <c r="D180" t="n">
+        <v>8.363393910532306</v>
+      </c>
+      <c r="E180" t="n">
+        <v>3505.969902752497</v>
+      </c>
+      <c r="F180" t="n">
+        <v>977.1692635698893</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>002-1638-R</t>
+        </is>
+      </c>
+      <c r="B181" t="n">
+        <v>2002</v>
+      </c>
+      <c r="C181" t="n">
+        <v>186.9355924865863</v>
+      </c>
+      <c r="D181" t="n">
+        <v>4.559474035900823</v>
+      </c>
+      <c r="E181" t="n">
+        <v>1192.601553103073</v>
+      </c>
+      <c r="F181" t="n">
+        <v>803.9526811440414</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>002-1638-R</t>
+        </is>
+      </c>
+      <c r="B182" t="n">
+        <v>2003</v>
+      </c>
+      <c r="C182" t="n">
+        <v>237.9443037455086</v>
+      </c>
+      <c r="D182" t="n">
+        <v>4.151446166044652</v>
+      </c>
+      <c r="E182" t="n">
+        <v>1267.836786259809</v>
+      </c>
+      <c r="F182" t="n">
+        <v>824.7500032227753</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>002-1638-R</t>
+        </is>
+      </c>
+      <c r="B183" t="n">
+        <v>2004</v>
+      </c>
+      <c r="C183" t="n">
+        <v>282.7409078831396</v>
+      </c>
+      <c r="D183" t="n">
+        <v>7.024618791319742</v>
+      </c>
+      <c r="E183" t="n">
+        <v>1513.496712120587</v>
+      </c>
+      <c r="F183" t="n">
+        <v>985.3322592379582</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>002-1638-R</t>
+        </is>
+      </c>
+      <c r="B184" t="n">
+        <v>2005</v>
+      </c>
+      <c r="C184" t="n">
+        <v>260.4351093601117</v>
+      </c>
+      <c r="D184" t="n">
+        <v>5.96056506394152</v>
+      </c>
+      <c r="E184" t="n">
+        <v>1952.914209770202</v>
+      </c>
+      <c r="F184" t="n">
+        <v>811.1675350918348</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>002-1638-R</t>
+        </is>
+      </c>
+      <c r="B185" t="n">
+        <v>2006</v>
+      </c>
+      <c r="C185" t="n">
+        <v>261.2300812649387</v>
+      </c>
+      <c r="D185" t="n">
+        <v>8.94932208499943</v>
+      </c>
+      <c r="E185" t="n">
+        <v>2914.322446532713</v>
+      </c>
+      <c r="F185" t="n">
+        <v>1246.44043758715</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>002-1638-R</t>
+        </is>
+      </c>
+      <c r="B186" t="n">
+        <v>2008</v>
+      </c>
+      <c r="C186" t="n">
+        <v>265.9655627457725</v>
+      </c>
+      <c r="D186" t="n">
+        <v>13.25419081423214</v>
+      </c>
+      <c r="E186" t="n">
+        <v>3882.618104621513</v>
+      </c>
+      <c r="F186" t="n">
+        <v>1343.326091095871</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>002-1638-R</t>
+        </is>
+      </c>
+      <c r="B187" t="n">
+        <v>2010</v>
+      </c>
+      <c r="C187" t="n">
+        <v>188.740936951179</v>
+      </c>
+      <c r="D187" t="n">
+        <v>4.810128547269732</v>
+      </c>
+      <c r="E187" t="n">
+        <v>2043.760149084331</v>
+      </c>
+      <c r="F187" t="n">
+        <v>826.5717141899352</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>002-1638-R</t>
+        </is>
+      </c>
+      <c r="B188" t="n">
+        <v>2011</v>
+      </c>
+      <c r="C188" t="n">
+        <v>256.7366468616509</v>
+      </c>
+      <c r="D188" t="n">
+        <v>18.54963244292455</v>
+      </c>
+      <c r="E188" t="n">
+        <v>10528.90858339543</v>
+      </c>
+      <c r="F188" t="n">
+        <v>1482.354586999677</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>002-1638-R</t>
+        </is>
+      </c>
+      <c r="B189" t="n">
+        <v>2012</v>
+      </c>
+      <c r="C189" t="n">
+        <v>280.7240502987199</v>
+      </c>
+      <c r="D189" t="n">
+        <v>9.817256696488759</v>
+      </c>
+      <c r="E189" t="n">
+        <v>5320.726892220153</v>
+      </c>
+      <c r="F189" t="n">
+        <v>1337.501895882453</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>002-1638-R</t>
+        </is>
+      </c>
+      <c r="B190" t="n">
+        <v>2013</v>
+      </c>
+      <c r="C190" t="n">
+        <v>279.5106688300704</v>
+      </c>
+      <c r="D190" t="n">
+        <v>19.61633942118484</v>
+      </c>
+      <c r="E190" t="n">
+        <v>14273.98569047706</v>
+      </c>
+      <c r="F190" t="n">
+        <v>1369.144592361439</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>002-1638-R</t>
+        </is>
+      </c>
+      <c r="B191" t="n">
+        <v>2015</v>
+      </c>
+      <c r="C191" t="n">
+        <v>281.391781661804</v>
+      </c>
+      <c r="D191" t="n">
+        <v>6.919611375126133</v>
+      </c>
+      <c r="E191" t="n">
+        <v>3160.05044952898</v>
+      </c>
+      <c r="F191" t="n">
+        <v>1814.596068371525</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>002-1638-R</t>
+        </is>
+      </c>
+      <c r="B192" t="n">
+        <v>2016</v>
+      </c>
+      <c r="C192" t="n">
+        <v>193.5739349988294</v>
+      </c>
+      <c r="D192" t="n">
+        <v>4.615766964464658</v>
+      </c>
+      <c r="E192" t="n">
+        <v>2117.966123631714</v>
+      </c>
+      <c r="F192" t="n">
+        <v>1169.255413566833</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>002-1638-R</t>
+        </is>
+      </c>
+      <c r="B193" t="n">
+        <v>2017</v>
+      </c>
+      <c r="C193" t="n">
+        <v>258.0705993943514</v>
+      </c>
+      <c r="D193" t="n">
+        <v>6.676136012961517</v>
+      </c>
+      <c r="E193" t="n">
+        <v>2556.496479314575</v>
+      </c>
+      <c r="F193" t="inlineStr"/>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>002-1638-R</t>
+        </is>
+      </c>
+      <c r="B194" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C194" t="n">
+        <v>311.9461705658915</v>
+      </c>
+      <c r="D194" t="n">
+        <v>11.599703202163</v>
+      </c>
+      <c r="E194" t="n">
+        <v>6344.142210842683</v>
+      </c>
+      <c r="F194" t="inlineStr"/>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>002-1638-R</t>
+        </is>
+      </c>
+      <c r="B195" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C195" t="n">
+        <v>359.609647881713</v>
+      </c>
+      <c r="D195" t="n">
+        <v>23.97881045961056</v>
+      </c>
+      <c r="E195" t="n">
+        <v>10217.66999692768</v>
+      </c>
+      <c r="F195" t="n">
+        <v>2828.922007046827</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>002-1638-R</t>
+        </is>
+      </c>
+      <c r="B196" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C196" t="n">
+        <v>275.8758258031834</v>
+      </c>
+      <c r="D196" t="n">
+        <v>7.772071238083376</v>
+      </c>
+      <c r="E196" t="n">
+        <v>2042.444106610554</v>
+      </c>
+      <c r="F196" t="n">
+        <v>2836.448730087902</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>002-1638-R</t>
+        </is>
+      </c>
+      <c r="B197" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C197" t="n">
+        <v>308.8526107116525</v>
+      </c>
+      <c r="D197" t="n">
+        <v>12.0831447480245</v>
+      </c>
+      <c r="E197" t="n">
+        <v>4281.316022826906</v>
+      </c>
+      <c r="F197" t="n">
+        <v>2664.530189270934</v>
       </c>
     </row>
   </sheetData>
@@ -4198,7 +4722,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4251,17 +4775,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Leira</t>
+          <t>Nitelva</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>002-3384-R</t>
+          <t>002-1638-R</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Leira nedstrøms Krokfoss</t>
+          <t>Nitelva Slattum-Kjeller</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -4271,36 +4795,36 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>no trend</t>
+          <t>increasing</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0.2168604205660558</v>
+        <v>0.003706522671735435</v>
       </c>
       <c r="G2" t="n">
-        <v>2.26013652149758</v>
+        <v>3.312790442485195</v>
       </c>
       <c r="H2" t="n">
-        <v>5.714852691026019</v>
+        <v>4.742333793851008</v>
       </c>
       <c r="I2" t="n">
-        <v>-1.074212141792748</v>
+        <v>1.843484461886931</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Leira</t>
+          <t>Nitelva</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>002-3384-R</t>
+          <t>002-1638-R</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Leira nedstrøms Krokfoss</t>
+          <t>Nitelva Slattum-Kjeller</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -4314,32 +4838,32 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0.05681822931485225</v>
+        <v>0.14334161203712</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.7138617998550546</v>
+        <v>0.1381047748806674</v>
       </c>
       <c r="H3" t="n">
-        <v>0.01805823905930397</v>
+        <v>0.3776999324752307</v>
       </c>
       <c r="I3" t="n">
-        <v>-1.432259895096275</v>
+        <v>-0.07319037913797777</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Leira</t>
+          <t>Nitelva</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>002-3384-R</t>
+          <t>002-1638-R</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Leira nedstrøms Krokfoss</t>
+          <t>Nitelva Slattum-Kjeller</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -4353,32 +4877,32 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>0.0638436989206157</v>
+        <v>0.3333582434882612</v>
       </c>
       <c r="G4" t="n">
-        <v>-532.6316209273488</v>
+        <v>50.33548671064586</v>
       </c>
       <c r="H4" t="n">
-        <v>24.60413403172788</v>
+        <v>161.9822856247093</v>
       </c>
       <c r="I4" t="n">
-        <v>-1229.156479641246</v>
+        <v>-50.57992581489249</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Leira</t>
+          <t>Nitelva</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>002-3384-R</t>
+          <t>002-1638-R</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Leira nedstrøms Krokfoss</t>
+          <t>Nitelva Slattum-Kjeller</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -4392,32 +4916,32 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>0.01107437281616974</v>
+        <v>0.0003809525703206695</v>
       </c>
       <c r="G5" t="n">
-        <v>37.86135639566405</v>
+        <v>47.1828298825053</v>
       </c>
       <c r="H5" t="n">
-        <v>60.632630544393</v>
+        <v>73.36351850874109</v>
       </c>
       <c r="I5" t="n">
-        <v>6.974659534164441</v>
+        <v>21.21055431581912</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Gansåa</t>
+          <t>Leira</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>002-3655-R</t>
+          <t>002-3384-R</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Gansåa</t>
+          <t>Leira nedstrøms Krokfoss</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -4431,32 +4955,32 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>0.9015386266571279</v>
+        <v>0.2168604205660558</v>
       </c>
       <c r="G6" t="n">
-        <v>-0.05953038634484983</v>
+        <v>2.26013652149758</v>
       </c>
       <c r="H6" t="n">
-        <v>4.136771748209011</v>
+        <v>5.714852691026019</v>
       </c>
       <c r="I6" t="n">
-        <v>-2.209477343905624</v>
+        <v>-1.074212141792748</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Gansåa</t>
+          <t>Leira</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>002-3655-R</t>
+          <t>002-3384-R</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Gansåa</t>
+          <t>Leira nedstrøms Krokfoss</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -4470,32 +4994,32 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>0.2655103889538737</v>
+        <v>0.05681822931485225</v>
       </c>
       <c r="G7" t="n">
-        <v>0.04413910262544479</v>
+        <v>-0.7138617998550546</v>
       </c>
       <c r="H7" t="n">
-        <v>0.2304256015589452</v>
+        <v>0.01805823905930397</v>
       </c>
       <c r="I7" t="n">
-        <v>-0.1445079368444659</v>
+        <v>-1.432259895096275</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Gansåa</t>
+          <t>Leira</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>002-3655-R</t>
+          <t>002-3384-R</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Gansåa</t>
+          <t>Leira nedstrøms Krokfoss</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -4509,32 +5033,32 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>0.5361867719001741</v>
+        <v>0.0638436989206157</v>
       </c>
       <c r="G8" t="n">
-        <v>14.32235047283566</v>
+        <v>-532.6316209273488</v>
       </c>
       <c r="H8" t="n">
-        <v>87.55136360349167</v>
+        <v>24.60413403172788</v>
       </c>
       <c r="I8" t="n">
-        <v>-79.39285653432115</v>
+        <v>-1229.156479641246</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Gansåa</t>
+          <t>Leira</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>002-3655-R</t>
+          <t>002-3384-R</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Gansåa</t>
+          <t>Leira nedstrøms Krokfoss</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -4544,36 +5068,36 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>no trend</t>
+          <t>increasing</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>0.7105230229164894</v>
+        <v>0.01107437281616974</v>
       </c>
       <c r="G9" t="n">
-        <v>7.93848284846395</v>
+        <v>37.86135639566405</v>
       </c>
       <c r="H9" t="n">
-        <v>57.37197650008329</v>
+        <v>60.632630544393</v>
       </c>
       <c r="I9" t="n">
-        <v>-33.96071005019476</v>
+        <v>6.974659534164441</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Rømua</t>
+          <t>Gansåa</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>002-3659-R</t>
+          <t>002-3655-R</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Rømua</t>
+          <t>Gansåa</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -4587,32 +5111,32 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>0.7115714636761059</v>
+        <v>0.9015386266571279</v>
       </c>
       <c r="G10" t="n">
-        <v>0.9491311291513114</v>
+        <v>-0.05953038634484983</v>
       </c>
       <c r="H10" t="n">
-        <v>4.701286981629579</v>
+        <v>4.136771748209011</v>
       </c>
       <c r="I10" t="n">
-        <v>-3.015956783834657</v>
+        <v>-2.209477343905624</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Rømua</t>
+          <t>Gansåa</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>002-3659-R</t>
+          <t>002-3655-R</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Rømua</t>
+          <t>Gansåa</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -4626,32 +5150,32 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>0.4596078230489589</v>
+        <v>0.2655103889538737</v>
       </c>
       <c r="G11" t="n">
-        <v>0.1627969349867363</v>
+        <v>0.04413910262544479</v>
       </c>
       <c r="H11" t="n">
-        <v>0.3811676406768105</v>
+        <v>0.2304256015589452</v>
       </c>
       <c r="I11" t="n">
-        <v>-0.2588144939937264</v>
+        <v>-0.1445079368444659</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Rømua</t>
+          <t>Gansåa</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>002-3659-R</t>
+          <t>002-3655-R</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Rømua</t>
+          <t>Gansåa</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -4665,32 +5189,32 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>0.4922895298178107</v>
+        <v>0.5361867719001741</v>
       </c>
       <c r="G12" t="n">
-        <v>87.4589005140168</v>
+        <v>14.32235047283566</v>
       </c>
       <c r="H12" t="n">
-        <v>268.0822859933359</v>
+        <v>87.55136360349167</v>
       </c>
       <c r="I12" t="n">
-        <v>-175.1107357484751</v>
+        <v>-79.39285653432115</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Rømua</t>
+          <t>Gansåa</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>002-3659-R</t>
+          <t>002-3655-R</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Rømua</t>
+          <t>Gansåa</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -4700,36 +5224,36 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>increasing</t>
+          <t>no trend</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>0.02784675596413333</v>
+        <v>0.7105230229164894</v>
       </c>
       <c r="G13" t="n">
-        <v>17.66534290144933</v>
+        <v>7.93848284846395</v>
       </c>
       <c r="H13" t="n">
-        <v>33.16595563990364</v>
+        <v>57.37197650008329</v>
       </c>
       <c r="I13" t="n">
-        <v>4.251743122818753</v>
+        <v>-33.96071005019476</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Åa</t>
+          <t>Rømua</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>002-3685-R</t>
+          <t>002-3659-R</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Fossåa</t>
+          <t>Rømua</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -4743,32 +5267,32 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>0.7544541774940892</v>
+        <v>0.7115714636761059</v>
       </c>
       <c r="G14" t="n">
-        <v>-2.007104115609447</v>
+        <v>0.9491311291513114</v>
       </c>
       <c r="H14" t="n">
-        <v>7.136326473416968</v>
+        <v>4.701286981629579</v>
       </c>
       <c r="I14" t="n">
-        <v>-13.20097383556671</v>
+        <v>-3.015956783834657</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Åa</t>
+          <t>Rømua</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>002-3685-R</t>
+          <t>002-3659-R</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Fossåa</t>
+          <t>Rømua</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -4782,32 +5306,32 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>0.7544541774940892</v>
+        <v>0.4596078230489589</v>
       </c>
       <c r="G15" t="n">
-        <v>0.1427993344868685</v>
+        <v>0.1627969349867363</v>
       </c>
       <c r="H15" t="n">
-        <v>1.136789423141088</v>
+        <v>0.3811676406768105</v>
       </c>
       <c r="I15" t="n">
-        <v>-0.4775133286467552</v>
+        <v>-0.2588144939937264</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Åa</t>
+          <t>Rømua</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>002-3685-R</t>
+          <t>002-3659-R</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Fossåa</t>
+          <t>Rømua</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -4821,32 +5345,32 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>0.6021675277481957</v>
+        <v>0.4922895298178107</v>
       </c>
       <c r="G16" t="n">
-        <v>289.4495655586229</v>
+        <v>87.4589005140168</v>
       </c>
       <c r="H16" t="n">
-        <v>685.7418448572769</v>
+        <v>268.0822859933359</v>
       </c>
       <c r="I16" t="n">
-        <v>-320.1356694985707</v>
+        <v>-175.1107357484751</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Åa</t>
+          <t>Rømua</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>002-3685-R</t>
+          <t>002-3659-R</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Fossåa</t>
+          <t>Rømua</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -4856,36 +5380,36 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>no trend</t>
+          <t>increasing</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>0.9169652366288645</v>
+        <v>0.02784675596413333</v>
       </c>
       <c r="G17" t="n">
-        <v>-15.83703837667097</v>
+        <v>17.66534290144933</v>
       </c>
       <c r="H17" t="n">
-        <v>132.9925757844316</v>
+        <v>33.16595563990364</v>
       </c>
       <c r="I17" t="n">
-        <v>-85.63918220144831</v>
+        <v>4.251743122818753</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Nitelva</t>
+          <t>Åa</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>002-3891-R</t>
+          <t>002-3685-R</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Nedre Nitelva</t>
+          <t>Fossåa</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -4899,32 +5423,32 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>0.9062974979468705</v>
+        <v>0.7544541774940892</v>
       </c>
       <c r="G18" t="n">
-        <v>0.2817002539394301</v>
+        <v>-2.007104115609447</v>
       </c>
       <c r="H18" t="n">
-        <v>4.255084072200583</v>
+        <v>7.136326473416968</v>
       </c>
       <c r="I18" t="n">
-        <v>-4.495242012266324</v>
+        <v>-13.20097383556671</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Nitelva</t>
+          <t>Åa</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>002-3891-R</t>
+          <t>002-3685-R</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Nedre Nitelva</t>
+          <t>Fossåa</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -4938,32 +5462,32 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>0.2894224860302206</v>
+        <v>0.7544541774940892</v>
       </c>
       <c r="G19" t="n">
-        <v>-0.1096013510329925</v>
+        <v>0.1427993344868685</v>
       </c>
       <c r="H19" t="n">
-        <v>0.1021467846264608</v>
+        <v>1.136789423141088</v>
       </c>
       <c r="I19" t="n">
-        <v>-0.3779863621768961</v>
+        <v>-0.4775133286467552</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Nitelva</t>
+          <t>Åa</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>002-3891-R</t>
+          <t>002-3685-R</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Nedre Nitelva</t>
+          <t>Fossåa</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -4977,32 +5501,32 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>0.07824219874308347</v>
+        <v>0.6021675277481957</v>
       </c>
       <c r="G20" t="n">
-        <v>-69.26780295870621</v>
+        <v>289.4495655586229</v>
       </c>
       <c r="H20" t="n">
-        <v>10.96226035007863</v>
+        <v>685.7418448572769</v>
       </c>
       <c r="I20" t="n">
-        <v>-136.0914998271753</v>
+        <v>-320.1356694985707</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Nitelva</t>
+          <t>Åa</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>002-3891-R</t>
+          <t>002-3685-R</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Nedre Nitelva</t>
+          <t>Fossåa</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -5012,36 +5536,36 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>increasing</t>
+          <t>no trend</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>0.002858749184990295</v>
+        <v>0.9169652366288645</v>
       </c>
       <c r="G21" t="n">
-        <v>43.65557962837244</v>
+        <v>-15.83703837667097</v>
       </c>
       <c r="H21" t="n">
-        <v>63.93200172841765</v>
+        <v>132.9925757844316</v>
       </c>
       <c r="I21" t="n">
-        <v>15.5849051794357</v>
+        <v>-85.63918220144831</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Sagelva</t>
+          <t>Nitelva</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>002-3899-R</t>
+          <t>002-3891-R</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Fjellhamarelva - Sagelva</t>
+          <t>Nedre Nitelva</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -5055,32 +5579,32 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>0.7481053914270006</v>
+        <v>0.9062974979468705</v>
       </c>
       <c r="G22" t="n">
-        <v>0.1374811663549445</v>
+        <v>0.2817002539394301</v>
       </c>
       <c r="H22" t="n">
-        <v>0.7441654612608859</v>
+        <v>4.255084072200583</v>
       </c>
       <c r="I22" t="n">
-        <v>-0.4775340659607014</v>
+        <v>-4.495242012266324</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Sagelva</t>
+          <t>Nitelva</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>002-3899-R</t>
+          <t>002-3891-R</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Fjellhamarelva - Sagelva</t>
+          <t>Nedre Nitelva</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -5094,32 +5618,32 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>0.2117118319412423</v>
+        <v>0.2894224860302206</v>
       </c>
       <c r="G23" t="n">
-        <v>0.0218681131362306</v>
+        <v>-0.1096013510329925</v>
       </c>
       <c r="H23" t="n">
-        <v>0.06376835757875088</v>
+        <v>0.1021467846264608</v>
       </c>
       <c r="I23" t="n">
-        <v>-0.01275880990492734</v>
+        <v>-0.3779863621768961</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Sagelva</t>
+          <t>Nitelva</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>002-3899-R</t>
+          <t>002-3891-R</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Fjellhamarelva - Sagelva</t>
+          <t>Nedre Nitelva</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -5133,32 +5657,32 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>0.5206932698330875</v>
+        <v>0.07824219874308347</v>
       </c>
       <c r="G24" t="n">
-        <v>5.700273546929941</v>
+        <v>-69.26780295870621</v>
       </c>
       <c r="H24" t="n">
-        <v>23.68467715206089</v>
+        <v>10.96226035007863</v>
       </c>
       <c r="I24" t="n">
-        <v>-11.53220793306063</v>
+        <v>-136.0914998271753</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Sagelva</t>
+          <t>Nitelva</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>002-3899-R</t>
+          <t>002-3891-R</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Fjellhamarelva - Sagelva</t>
+          <t>Nedre Nitelva</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -5172,32 +5696,32 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>0.004782669315397836</v>
+        <v>0.002858749184990295</v>
       </c>
       <c r="G25" t="n">
-        <v>9.282071767869864</v>
+        <v>43.65557962837244</v>
       </c>
       <c r="H25" t="n">
-        <v>14.60383702754566</v>
+        <v>63.93200172841765</v>
       </c>
       <c r="I25" t="n">
-        <v>2.785257145737035</v>
+        <v>15.5849051794357</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Jeksla</t>
+          <t>Sagelva</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>002-599-R</t>
+          <t>002-3899-R</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Jeksla</t>
+          <t>Fjellhamarelva - Sagelva</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -5211,32 +5735,32 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>0.1143167755404042</v>
+        <v>0.7481053914270006</v>
       </c>
       <c r="G26" t="n">
-        <v>-0.2987765680358331</v>
+        <v>0.1374811663549445</v>
       </c>
       <c r="H26" t="n">
-        <v>0.0716498597037252</v>
+        <v>0.7441654612608859</v>
       </c>
       <c r="I26" t="n">
-        <v>-0.7122935207863031</v>
+        <v>-0.4775340659607014</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Jeksla</t>
+          <t>Sagelva</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>002-599-R</t>
+          <t>002-3899-R</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Jeksla</t>
+          <t>Fjellhamarelva - Sagelva</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -5250,32 +5774,32 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>0.5727823105937271</v>
+        <v>0.2117118319412423</v>
       </c>
       <c r="G27" t="n">
-        <v>-0.007690429796718981</v>
+        <v>0.0218681131362306</v>
       </c>
       <c r="H27" t="n">
-        <v>0.01847104236896741</v>
+        <v>0.06376835757875088</v>
       </c>
       <c r="I27" t="n">
-        <v>-0.03838859060596889</v>
+        <v>-0.01275880990492734</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Jeksla</t>
+          <t>Sagelva</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>002-599-R</t>
+          <t>002-3899-R</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Jeksla</t>
+          <t>Fjellhamarelva - Sagelva</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -5289,54 +5813,210 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>0.9741177473553713</v>
+        <v>0.5206932698330875</v>
       </c>
       <c r="G28" t="n">
-        <v>-0.6604755791175183</v>
+        <v>5.700273546929941</v>
       </c>
       <c r="H28" t="n">
-        <v>15.07081259248431</v>
+        <v>23.68467715206089</v>
       </c>
       <c r="I28" t="n">
-        <v>-23.55880784620273</v>
+        <v>-11.53220793306063</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
+          <t>Sagelva</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>002-3899-R</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Fjellhamarelva - Sagelva</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>TOC_tonn</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>increasing</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>0.004782669315397836</v>
+      </c>
+      <c r="G29" t="n">
+        <v>9.282071767869864</v>
+      </c>
+      <c r="H29" t="n">
+        <v>14.60383702754566</v>
+      </c>
+      <c r="I29" t="n">
+        <v>2.785257145737035</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
           <t>Jeksla</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>002-599-R</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>Jeksla</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>TOTN_tonn</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>no trend</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>0.1143167755404042</v>
+      </c>
+      <c r="G30" t="n">
+        <v>-0.2987765680358331</v>
+      </c>
+      <c r="H30" t="n">
+        <v>0.0716498597037252</v>
+      </c>
+      <c r="I30" t="n">
+        <v>-0.7122935207863031</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Jeksla</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>002-599-R</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Jeksla</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>TOTP_tonn</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>no trend</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>0.5727823105937271</v>
+      </c>
+      <c r="G31" t="n">
+        <v>-0.007690429796718981</v>
+      </c>
+      <c r="H31" t="n">
+        <v>0.01847104236896741</v>
+      </c>
+      <c r="I31" t="n">
+        <v>-0.03838859060596889</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Jeksla</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>002-599-R</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Jeksla</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>SS_tonn</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>no trend</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>0.9741177473553713</v>
+      </c>
+      <c r="G32" t="n">
+        <v>-0.6604755791175183</v>
+      </c>
+      <c r="H32" t="n">
+        <v>15.07081259248431</v>
+      </c>
+      <c r="I32" t="n">
+        <v>-23.55880784620273</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Jeksla</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>002-599-R</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Jeksla</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
         <is>
           <t>TOC_tonn</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E33" t="inlineStr">
         <is>
           <t>no trend</t>
         </is>
       </c>
-      <c r="F29" t="n">
+      <c r="F33" t="n">
         <v>0.2241343019601669</v>
       </c>
-      <c r="G29" t="n">
+      <c r="G33" t="n">
         <v>1.309048991643165</v>
       </c>
-      <c r="H29" t="n">
+      <c r="H33" t="n">
         <v>3.858558727783756</v>
       </c>
-      <c r="I29" t="n">
+      <c r="I33" t="n">
         <v>-0.8642952039623104</v>
       </c>
     </row>

</xml_diff>